<commit_message>
feat: update APPRAISAL_rubric.xlsx and remove temporary file
</commit_message>
<xml_diff>
--- a/APPRAISAL_rubric.xlsx
+++ b/APPRAISAL_rubric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ageidv/ilo/deploy_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7994D4D2-253D-3245-B3D3-3254BFAEA9EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0CE3163-0055-E546-9DDD-77FB78432B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="25920" windowHeight="16380" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -896,7 +896,7 @@
     <t>TARJETA DE VALORACIÓN DE EVALUABILIDAD</t>
   </si>
   <si>
-    <t>4.1 ¿La teoría del cambio (por ejemplo, la expectativa de cómo ocurrirá el cambio) está claramente expresada y expuesta explícitamente de una manera que parezca plausible para el no especialista, en la narrativa y / o como un gráfico?Los productos parecen suficientes para el probable logro de resultados. La contribución esperada de los resultados al impacto también es clara?</t>
+    <t>¿Los productos del proyecto/programa/intervención son  suficientes para el logro de resultados previstos en la teoría del cambio  del proyecto?</t>
   </si>
 </sst>
 </file>
@@ -1245,9 +1245,6 @@
   </cellStyleXfs>
   <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1366,6 +1363,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2884,7 +2884,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="9.1640625" style="2"/>
+    <col min="1" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.625" header="0.511811023622047" footer="0.3"/>
@@ -2906,35 +2906,35 @@
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
     <col min="2" max="2" width="54.1640625" customWidth="1"/>
-    <col min="3" max="3" width="82.1640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="82.1640625" style="2" customWidth="1"/>
     <col min="16380" max="16384" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5 16380:16382" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5 16380:16382" s="11" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:5 16380:16382" s="10" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E2"/>
@@ -2942,17 +2942,17 @@
       <c r="XFA2"/>
       <c r="XFB2"/>
     </row>
-    <row r="3" spans="1:5 16380:16382" s="11" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A3" s="8" t="s">
+    <row r="3" spans="1:5 16380:16382" s="10" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E3"/>
@@ -2960,17 +2960,17 @@
       <c r="XFA3"/>
       <c r="XFB3"/>
     </row>
-    <row r="4" spans="1:5 16380:16382" s="11" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A4" s="8" t="s">
+    <row r="4" spans="1:5 16380:16382" s="10" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E4"/>
@@ -2978,17 +2978,17 @@
       <c r="XFA4"/>
       <c r="XFB4"/>
     </row>
-    <row r="5" spans="1:5 16380:16382" s="11" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
+    <row r="5" spans="1:5 16380:16382" s="10" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E5"/>
@@ -2997,184 +2997,184 @@
       <c r="XFB5"/>
     </row>
     <row r="6" spans="1:5 16380:16382" ht="48" x14ac:dyDescent="0.2">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5 16380:16382" ht="32" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:5 16380:16382" ht="80" x14ac:dyDescent="0.2">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:5 16380:16382" ht="80" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:5 16380:16382" ht="48" x14ac:dyDescent="0.2">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:5 16380:16382" ht="48" x14ac:dyDescent="0.2">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:5 16380:16382" ht="48" x14ac:dyDescent="0.2">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:5 16380:16382" ht="64" x14ac:dyDescent="0.2">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:5 16380:16382" ht="32" x14ac:dyDescent="0.2">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:5 16380:16382" ht="90" x14ac:dyDescent="0.2">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:5 16380:16382" ht="64" x14ac:dyDescent="0.2">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="9" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:5 16380:16382" ht="48" x14ac:dyDescent="0.2">
-      <c r="A17" s="20" t="s">
+      <c r="A17" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:5 16380:16382" s="11" customFormat="1" ht="68" x14ac:dyDescent="0.2">
-      <c r="A18" s="23" t="s">
+    <row r="18" spans="1:5 16380:16382" s="10" customFormat="1" ht="68" x14ac:dyDescent="0.2">
+      <c r="A18" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="9" t="s">
         <v>71</v>
       </c>
       <c r="E18"/>
@@ -3182,17 +3182,17 @@
       <c r="XFA18"/>
       <c r="XFB18"/>
     </row>
-    <row r="19" spans="1:5 16380:16382" s="11" customFormat="1" ht="68" x14ac:dyDescent="0.2">
-      <c r="A19" s="23" t="s">
+    <row r="19" spans="1:5 16380:16382" s="10" customFormat="1" ht="68" x14ac:dyDescent="0.2">
+      <c r="A19" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="9" t="s">
         <v>75</v>
       </c>
       <c r="E19"/>
@@ -3200,17 +3200,17 @@
       <c r="XFA19"/>
       <c r="XFB19"/>
     </row>
-    <row r="20" spans="1:5 16380:16382" s="11" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A20" s="23" t="s">
+    <row r="20" spans="1:5 16380:16382" s="10" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A20" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>79</v>
       </c>
       <c r="E20"/>
@@ -3218,17 +3218,17 @@
       <c r="XFA20"/>
       <c r="XFB20"/>
     </row>
-    <row r="21" spans="1:5 16380:16382" s="11" customFormat="1" ht="85" x14ac:dyDescent="0.2">
-      <c r="A21" s="27" t="s">
+    <row r="21" spans="1:5 16380:16382" s="10" customFormat="1" ht="85" x14ac:dyDescent="0.2">
+      <c r="A21" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="9" t="s">
         <v>83</v>
       </c>
       <c r="E21"/>
@@ -3236,17 +3236,17 @@
       <c r="XFA21"/>
       <c r="XFB21"/>
     </row>
-    <row r="22" spans="1:5 16380:16382" s="11" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A22" s="27" t="s">
+    <row r="22" spans="1:5 16380:16382" s="10" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A22" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="9" t="s">
         <v>87</v>
       </c>
       <c r="E22"/>
@@ -3254,17 +3254,17 @@
       <c r="XFA22"/>
       <c r="XFB22"/>
     </row>
-    <row r="23" spans="1:5 16380:16382" s="11" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A23" s="27" t="s">
+    <row r="23" spans="1:5 16380:16382" s="10" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A23" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="9" t="s">
         <v>91</v>
       </c>
       <c r="E23"/>
@@ -3273,628 +3273,628 @@
       <c r="XFB23"/>
     </row>
     <row r="24" spans="1:5 16380:16382" ht="80" x14ac:dyDescent="0.2">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="30" t="s">
+      <c r="B24" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="9" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:5 16380:16382" ht="96" x14ac:dyDescent="0.2">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="9" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:5 16380:16382" ht="64" x14ac:dyDescent="0.2">
-      <c r="A26" s="15" t="s">
+      <c r="A26" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="B26" s="16" t="s">
+      <c r="B26" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="9" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:5 16380:16382" ht="80" x14ac:dyDescent="0.2">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="9" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:5 16380:16382" ht="64" x14ac:dyDescent="0.2">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="9" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="29" spans="1:5 16380:16382" ht="64" x14ac:dyDescent="0.2">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="9" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="30" spans="1:5 16380:16382" ht="80" x14ac:dyDescent="0.2">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="9" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:5 16380:16382" ht="96" x14ac:dyDescent="0.2">
-      <c r="A31" s="32" t="s">
+      <c r="A31" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" s="9" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="32" spans="1:5 16380:16382" ht="64" x14ac:dyDescent="0.2">
-      <c r="A32" s="32" t="s">
+    <row r="32" spans="1:5 16380:16382" ht="45" x14ac:dyDescent="0.2">
+      <c r="A32" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="9" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A33" s="32" t="s">
+      <c r="A33" s="31" t="s">
         <v>127</v>
       </c>
-      <c r="B33" s="33" t="s">
+      <c r="B33" s="32" t="s">
         <v>128</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="9" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="64" x14ac:dyDescent="0.2">
-      <c r="A34" s="32" t="s">
+      <c r="A34" s="31" t="s">
         <v>131</v>
       </c>
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D34" s="9" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="96" x14ac:dyDescent="0.2">
-      <c r="A35" s="32" t="s">
+      <c r="A35" s="31" t="s">
         <v>135</v>
       </c>
-      <c r="B35" s="18" t="s">
+      <c r="B35" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="9" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A36" s="32" t="s">
+      <c r="A36" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="B36" s="34" t="s">
+      <c r="B36" s="33" t="s">
         <v>140</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="9" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A37" s="32" t="s">
+      <c r="A37" s="31" t="s">
         <v>143</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="9" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A38" s="32" t="s">
+      <c r="A38" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="B38" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" s="9" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="B39" s="16" t="s">
+      <c r="B39" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="9" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A40" s="15"/>
-      <c r="B40" s="18" t="s">
+      <c r="A40" s="14"/>
+      <c r="B40" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="9" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A41" s="35" t="s">
+      <c r="A41" s="34" t="s">
         <v>157</v>
       </c>
-      <c r="B41" s="16" t="s">
+      <c r="B41" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="9" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A42" s="35" t="s">
+      <c r="A42" s="34" t="s">
         <v>161</v>
       </c>
-      <c r="B42" s="17" t="s">
+      <c r="B42" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" s="9" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A43" s="35" t="s">
+      <c r="A43" s="34" t="s">
         <v>165</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="B43" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="D43" s="10" t="s">
+      <c r="D43" s="9" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A44" s="35" t="s">
+      <c r="A44" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="B44" s="18" t="s">
+      <c r="B44" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D44" s="9" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="120" x14ac:dyDescent="0.2">
-      <c r="A45" s="36" t="s">
+      <c r="A45" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="B45" s="30" t="s">
+      <c r="B45" s="29" t="s">
         <v>174</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="D45" s="9" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="96" x14ac:dyDescent="0.2">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="35" t="s">
         <v>177</v>
       </c>
-      <c r="B46" s="22" t="s">
+      <c r="B46" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="D46" s="9" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="75" x14ac:dyDescent="0.2">
-      <c r="A47" s="36" t="s">
+      <c r="A47" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="B47" s="22" t="s">
+      <c r="B47" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="D47" s="10" t="s">
+      <c r="D47" s="9" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="120" x14ac:dyDescent="0.2">
-      <c r="A48" s="36" t="s">
+      <c r="A48" s="35" t="s">
         <v>185</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="B48" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D48" s="10" t="s">
+      <c r="D48" s="9" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="90" x14ac:dyDescent="0.2">
-      <c r="A49" s="36" t="s">
+      <c r="A49" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="B49" s="31" t="s">
+      <c r="B49" s="30" t="s">
         <v>190</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="D49" s="10" t="s">
+      <c r="D49" s="9" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="105" x14ac:dyDescent="0.2">
-      <c r="A50" s="37" t="s">
+      <c r="A50" s="36" t="s">
         <v>193</v>
       </c>
-      <c r="B50" s="38" t="s">
+      <c r="B50" s="37" t="s">
         <v>194</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="D50" s="10" t="s">
+      <c r="D50" s="9" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A51" s="37" t="s">
+      <c r="A51" s="36" t="s">
         <v>197</v>
       </c>
-      <c r="B51" s="22" t="s">
+      <c r="B51" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="D51" s="10" t="s">
+      <c r="D51" s="9" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A52" s="32" t="s">
+      <c r="A52" s="31" t="s">
         <v>201</v>
       </c>
-      <c r="B52" s="16" t="s">
+      <c r="B52" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="D52" s="10" t="s">
+      <c r="D52" s="9" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A53" s="32"/>
-      <c r="B53" s="18" t="s">
+      <c r="A53" s="31"/>
+      <c r="B53" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="C53" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="D53" s="10" t="s">
+      <c r="D53" s="9" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="75" x14ac:dyDescent="0.2">
-      <c r="A54" s="15" t="s">
+      <c r="A54" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="B54" s="30" t="s">
+      <c r="B54" s="29" t="s">
         <v>208</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="C54" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="D54" s="10" t="s">
+      <c r="D54" s="9" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="60" x14ac:dyDescent="0.2">
-      <c r="A55" s="15" t="s">
+      <c r="A55" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="B55" s="17" t="s">
+      <c r="B55" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="C55" s="6" t="s">
+      <c r="C55" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="D55" s="10" t="s">
+      <c r="D55" s="9" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A56" s="15" t="s">
+      <c r="A56" s="14" t="s">
         <v>215</v>
       </c>
-      <c r="B56" s="17" t="s">
+      <c r="B56" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D56" s="10" t="s">
+      <c r="D56" s="9" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A57" s="15" t="s">
+      <c r="A57" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="B57" s="18" t="s">
+      <c r="B57" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="D57" s="10" t="s">
+      <c r="D57" s="9" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" x14ac:dyDescent="0.2">
-      <c r="A58" s="15" t="s">
+      <c r="A58" s="14" t="s">
         <v>223</v>
       </c>
-      <c r="B58" s="16" t="s">
+      <c r="B58" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="C58" s="6" t="s">
+      <c r="C58" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="D58" s="10" t="s">
+      <c r="D58" s="9" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A59" s="15" t="s">
+      <c r="A59" s="14" t="s">
         <v>227</v>
       </c>
-      <c r="B59" s="17" t="s">
+      <c r="B59" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D59" s="10" t="s">
+      <c r="D59" s="9" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A60" s="15" t="s">
+      <c r="A60" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="B60" s="39" t="s">
+      <c r="B60" s="38" t="s">
         <v>232</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="D60" s="10" t="s">
+      <c r="D60" s="9" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A61" s="15" t="s">
+      <c r="A61" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="B61" s="17" t="s">
+      <c r="B61" s="16" t="s">
         <v>236</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="D61" s="10" t="s">
+      <c r="D61" s="9" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A62" s="15" t="s">
+      <c r="A62" s="14" t="s">
         <v>239</v>
       </c>
-      <c r="B62" s="18" t="s">
+      <c r="B62" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="C62" s="6" t="s">
+      <c r="C62" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="D62" s="10" t="s">
+      <c r="D62" s="9" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A63" s="15" t="s">
+      <c r="A63" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="B63" s="40" t="s">
+      <c r="B63" s="39" t="s">
         <v>244</v>
       </c>
-      <c r="C63" s="6" t="s">
+      <c r="C63" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="D63" s="10" t="s">
+      <c r="D63" s="9" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A64" s="15" t="s">
+      <c r="A64" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="B64" s="16" t="s">
+      <c r="B64" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="C64" s="6" t="s">
+      <c r="C64" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="D64" s="10" t="s">
+      <c r="D64" s="9" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A65" s="15" t="s">
+      <c r="A65" s="14" t="s">
         <v>251</v>
       </c>
-      <c r="B65" s="17" t="s">
+      <c r="B65" s="16" t="s">
         <v>252</v>
       </c>
-      <c r="C65" s="6" t="s">
+      <c r="C65" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="D65" s="10" t="s">
+      <c r="D65" s="9" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A66" s="15" t="s">
+      <c r="A66" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="B66" s="18" t="s">
+      <c r="B66" s="17" t="s">
         <v>256</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="D66" s="9" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A67" s="35" t="s">
+      <c r="A67" s="34" t="s">
         <v>259</v>
       </c>
-      <c r="B67" s="41" t="s">
+      <c r="B67" s="40" t="s">
         <v>260</v>
       </c>
-      <c r="C67" s="6" t="s">
+      <c r="C67" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="D67" s="10" t="s">
+      <c r="D67" s="9" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A68" s="35" t="s">
+      <c r="A68" s="34" t="s">
         <v>263</v>
       </c>
-      <c r="B68" s="41" t="s">
+      <c r="B68" s="40" t="s">
         <v>264</v>
       </c>
-      <c r="C68" s="6" t="s">
+      <c r="C68" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="D68" s="10" t="s">
+      <c r="D68" s="9" t="s">
         <v>266</v>
       </c>
     </row>
@@ -3913,47 +3913,47 @@
   <dimension ref="B2:Q3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.5" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="9.1640625" style="2"/>
+    <col min="1" max="1" width="11.5" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:17" ht="63" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="42"/>
-      <c r="C2" s="1" t="s">
+      <c r="B2" s="41"/>
+      <c r="C2" s="42" t="s">
         <v>267</v>
       </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
     </row>
     <row r="3" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="42"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="42"/>
+      <c r="O3" s="42"/>
+      <c r="P3" s="42"/>
+      <c r="Q3" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>